<commit_message>
written test case on Update address
</commit_message>
<xml_diff>
--- a/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
+++ b/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{F2D2FD1F-9E2E-47CD-B018-3D8613FCE4D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{169171C6-20E9-4068-A0CB-76AB62555CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Signup365" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="GeneratorInformation" sheetId="7" r:id="rId12"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A22:E30"/>
+  <oleSize ref="A45:G60"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="805">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="806">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -2460,6 +2460,9 @@
   </si>
   <si>
     <t>charlie44636</t>
+  </si>
+  <si>
+    <t>Email with valid format</t>
   </si>
 </sst>
 </file>
@@ -2834,16 +2837,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2869,7 +2871,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -2900,20 +2902,20 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
   <dimension ref="A1:H106"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" style="6" customWidth="1"/>
     <col min="2" max="2" width="25" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.33203125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.5546875" style="6" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="25.6640625" style="6" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="3" width="18.28515625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="23.5703125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" style="6" customWidth="1"/>
+    <col min="7" max="7" width="25.7109375" style="6" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>15</v>
       </c>
@@ -2930,7 +2932,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>390</v>
       </c>
@@ -2947,7 +2949,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>395</v>
       </c>
@@ -2964,7 +2966,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>399</v>
       </c>
@@ -2981,7 +2983,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>404</v>
       </c>
@@ -2998,7 +3000,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>407</v>
       </c>
@@ -3015,7 +3017,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>434</v>
       </c>
@@ -3023,12 +3025,12 @@
         <v>435</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" s="6" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>436</v>
       </c>
@@ -3045,7 +3047,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>439</v>
       </c>
@@ -3062,7 +3064,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>445</v>
       </c>
@@ -3079,7 +3081,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>444</v>
       </c>
@@ -3096,7 +3098,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="4" customFormat="1" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" s="4" customFormat="1" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>450</v>
       </c>
@@ -3119,7 +3121,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>454</v>
       </c>
@@ -3142,7 +3144,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="24" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>259</v>
       </c>
@@ -3150,12 +3152,12 @@
         <v>461</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B25" s="6" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="27" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>463</v>
       </c>
@@ -3172,7 +3174,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>468</v>
       </c>
@@ -3189,7 +3191,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="29" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>473</v>
       </c>
@@ -3197,7 +3199,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>470</v>
       </c>
@@ -3205,7 +3207,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="32" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>472</v>
       </c>
@@ -3225,7 +3227,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>474</v>
       </c>
@@ -3245,7 +3247,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="35" spans="1:8" s="4" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" s="4" customFormat="1" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>481</v>
       </c>
@@ -3271,7 +3273,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>483</v>
       </c>
@@ -3297,7 +3299,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>492</v>
       </c>
@@ -3305,7 +3307,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>493</v>
       </c>
@@ -3313,7 +3315,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="40" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>495</v>
       </c>
@@ -3327,7 +3329,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>496</v>
       </c>
@@ -3341,7 +3343,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="42" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>495</v>
       </c>
@@ -3355,7 +3357,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>500</v>
       </c>
@@ -3369,7 +3371,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="44" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>504</v>
       </c>
@@ -3383,7 +3385,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>508</v>
       </c>
@@ -3397,7 +3399,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="46" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>509</v>
       </c>
@@ -3411,7 +3413,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>510</v>
       </c>
@@ -3425,7 +3427,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="48" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>513</v>
       </c>
@@ -3439,7 +3441,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>514</v>
       </c>
@@ -3453,7 +3455,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>517</v>
       </c>
@@ -3467,7 +3469,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>518</v>
       </c>
@@ -3481,7 +3483,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="52" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>522</v>
       </c>
@@ -3495,7 +3497,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>523</v>
       </c>
@@ -3509,7 +3511,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="54" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>526</v>
       </c>
@@ -3523,7 +3525,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>534</v>
       </c>
@@ -3537,7 +3539,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="56" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>529</v>
       </c>
@@ -3551,7 +3553,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>535</v>
       </c>
@@ -3565,7 +3567,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="58" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>533</v>
       </c>
@@ -3579,7 +3581,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>536</v>
       </c>
@@ -3593,7 +3595,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="60" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>539</v>
       </c>
@@ -3610,7 +3612,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>540</v>
       </c>
@@ -3627,7 +3629,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="62" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>547</v>
       </c>
@@ -3644,7 +3646,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>543</v>
       </c>
@@ -3661,7 +3663,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="64" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>550</v>
       </c>
@@ -3675,7 +3677,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>551</v>
       </c>
@@ -3689,7 +3691,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="66" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>555</v>
       </c>
@@ -3703,7 +3705,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>557</v>
       </c>
@@ -3717,7 +3719,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="68" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>561</v>
       </c>
@@ -3731,7 +3733,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>562</v>
       </c>
@@ -3745,7 +3747,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="70" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
         <v>565</v>
       </c>
@@ -3762,7 +3764,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>566</v>
       </c>
@@ -3779,7 +3781,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="72" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
         <v>569</v>
       </c>
@@ -3805,7 +3807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>570</v>
       </c>
@@ -3831,7 +3833,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="74" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>578</v>
       </c>
@@ -3851,7 +3853,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>579</v>
       </c>
@@ -3871,7 +3873,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="76" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>584</v>
       </c>
@@ -3894,7 +3896,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>585</v>
       </c>
@@ -3917,12 +3919,12 @@
         <v>592</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A78" s="10" t="s">
         <v>593</v>
       </c>
     </row>
-    <row r="79" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>539</v>
       </c>
@@ -3936,7 +3938,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>594</v>
       </c>
@@ -3950,7 +3952,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="81" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>547</v>
       </c>
@@ -3964,7 +3966,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
         <v>598</v>
       </c>
@@ -3978,7 +3980,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="83" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>550</v>
       </c>
@@ -3992,7 +3994,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>602</v>
       </c>
@@ -4006,7 +4008,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="85" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>555</v>
       </c>
@@ -4020,7 +4022,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
         <v>606</v>
       </c>
@@ -4034,7 +4036,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="87" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>561</v>
       </c>
@@ -4048,7 +4050,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
         <v>613</v>
       </c>
@@ -4062,7 +4064,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="89" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
         <v>565</v>
       </c>
@@ -4076,7 +4078,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
         <v>614</v>
       </c>
@@ -4090,7 +4092,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="91" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>569</v>
       </c>
@@ -4113,7 +4115,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
         <v>619</v>
       </c>
@@ -4136,7 +4138,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="93" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>578</v>
       </c>
@@ -4153,7 +4155,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
         <v>624</v>
       </c>
@@ -4170,7 +4172,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="95" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
         <v>584</v>
       </c>
@@ -4193,7 +4195,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A96" s="6" t="s">
         <v>630</v>
       </c>
@@ -4216,12 +4218,12 @@
         <v>460</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A97" s="10" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="98" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>569</v>
       </c>
@@ -4244,7 +4246,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A99" s="6" t="s">
         <v>644</v>
       </c>
@@ -4267,7 +4269,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="100" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
         <v>578</v>
       </c>
@@ -4284,7 +4286,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A101" s="6" t="s">
         <v>649</v>
       </c>
@@ -4301,7 +4303,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="102" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:7" s="4" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
         <v>584</v>
       </c>
@@ -4324,7 +4326,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A103" s="6" t="s">
         <v>660</v>
       </c>
@@ -4347,7 +4349,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="105" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:7" s="4" customFormat="1" ht="28.9" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
         <v>663</v>
       </c>
@@ -4367,7 +4369,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:7" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A106" s="6" t="s">
         <v>667</v>
       </c>
@@ -4414,12 +4416,12 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91B8B5A6-41F7-4B76-9B90-A5C1587D6738}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -4427,7 +4429,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -4443,17 +4445,17 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B6D8AE-3776-4B30-9CCC-A0DDA74A5F86}">
   <dimension ref="A1:G47"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="34.21875" customWidth="1"/>
-    <col min="4" max="4" width="40.21875" customWidth="1"/>
-    <col min="5" max="5" width="38.6640625" customWidth="1"/>
-    <col min="6" max="6" width="40.5546875" customWidth="1"/>
-    <col min="7" max="7" width="33.109375" customWidth="1"/>
+    <col min="3" max="3" width="34.28515625" customWidth="1"/>
+    <col min="4" max="4" width="40.28515625" customWidth="1"/>
+    <col min="5" max="5" width="38.7109375" customWidth="1"/>
+    <col min="6" max="6" width="40.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -4461,7 +4463,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -4469,7 +4471,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -4480,7 +4482,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>674</v>
       </c>
@@ -4491,7 +4493,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -4505,7 +4507,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>678</v>
       </c>
@@ -4519,7 +4521,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
@@ -4533,7 +4535,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>682</v>
       </c>
@@ -4547,7 +4549,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -4561,7 +4563,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>686</v>
       </c>
@@ -4575,7 +4577,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>15</v>
       </c>
@@ -4598,7 +4600,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>693</v>
       </c>
@@ -4621,7 +4623,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -4644,7 +4646,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>273</v>
       </c>
@@ -4667,7 +4669,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="22" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>15</v>
       </c>
@@ -4687,7 +4689,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>705</v>
       </c>
@@ -4707,7 +4709,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="25" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>15</v>
       </c>
@@ -4721,7 +4723,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>711</v>
       </c>
@@ -4735,7 +4737,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="28" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>15</v>
       </c>
@@ -4749,7 +4751,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>714</v>
       </c>
@@ -4763,7 +4765,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="31" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>15</v>
       </c>
@@ -4777,7 +4779,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>715</v>
       </c>
@@ -4791,7 +4793,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="34" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>15</v>
       </c>
@@ -4805,7 +4807,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>716</v>
       </c>
@@ -4819,7 +4821,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="37" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>15</v>
       </c>
@@ -4833,7 +4835,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>718</v>
       </c>
@@ -4847,7 +4849,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="40" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>15</v>
       </c>
@@ -4863,8 +4865,11 @@
       <c r="E40" s="3" t="s">
         <v>721</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F40" s="3" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>722</v>
       </c>
@@ -4880,8 +4885,11 @@
       <c r="E41" t="s">
         <v>723</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F41" s="2" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>15</v>
       </c>
@@ -4901,7 +4909,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>725</v>
       </c>
@@ -4921,7 +4929,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="46" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
@@ -4941,7 +4949,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>118</v>
       </c>
@@ -4965,6 +4973,7 @@
   <hyperlinks>
     <hyperlink ref="E23" r:id="rId1" xr:uid="{4F8EBCF3-1866-4794-8F4F-9060DF8CC2E9}"/>
     <hyperlink ref="F23" r:id="rId2" xr:uid="{94686A13-7684-4DC8-AB87-C0C9E54E1546}"/>
+    <hyperlink ref="F41" r:id="rId3" xr:uid="{D4C7FB14-C4E4-42CA-8DE0-98E0B10DA5A6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4973,14 +4982,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77142416-745D-4F9D-B8CB-E786E8AF6BF4}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>77</v>
       </c>
@@ -4991,7 +5000,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>414</v>
       </c>
@@ -5002,7 +5011,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>803</v>
       </c>
@@ -5015,16 +5024,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7C6CDDE-28EE-4E4D-95AF-5786FC71BBC0}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -5041,7 +5050,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>80</v>
       </c>
@@ -5058,7 +5067,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -5082,7 +5091,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>422</v>
       </c>
@@ -5102,7 +5111,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -5118,7 +5127,7 @@
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>428</v>
       </c>
@@ -5126,7 +5135,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
@@ -5142,7 +5151,7 @@
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>431</v>
       </c>
@@ -5161,18 +5170,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB07B270-85DC-4F6D-8AC7-D93CAE493508}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.109375" style="11" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="17.33203125" style="11" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" style="11" customWidth="1"/>
-    <col min="5" max="5" width="16.77734375" style="11" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" style="11" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="11"/>
+    <col min="1" max="1" width="15.140625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" style="11" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" style="11" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" style="11" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" style="11" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="11" customWidth="1"/>
+    <col min="7" max="16384" width="8.85546875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>539</v>
       </c>
@@ -5189,7 +5198,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>732</v>
       </c>
@@ -5206,7 +5215,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="4" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
         <v>569</v>
       </c>
@@ -5226,7 +5235,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>740</v>
       </c>
@@ -5246,7 +5255,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="7" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>742</v>
       </c>
@@ -5254,7 +5263,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>743</v>
       </c>
@@ -5262,7 +5271,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="10" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
         <v>746</v>
       </c>
@@ -5270,12 +5279,12 @@
         <v>748</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="13" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>749</v>
       </c>
@@ -5295,7 +5304,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>750</v>
       </c>
@@ -5315,7 +5324,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="15" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
         <v>756</v>
       </c>
@@ -5332,7 +5341,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>759</v>
       </c>
@@ -5349,7 +5358,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="17" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>763</v>
       </c>
@@ -5366,7 +5375,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>765</v>
       </c>
@@ -5383,7 +5392,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
         <v>769</v>
       </c>
@@ -5391,7 +5400,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>771</v>
       </c>
@@ -5399,7 +5408,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>772</v>
       </c>
@@ -5416,7 +5425,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>773</v>
       </c>
@@ -5433,7 +5442,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="23" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>777</v>
       </c>
@@ -5450,7 +5459,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>778</v>
       </c>
@@ -5467,7 +5476,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="25" spans="1:7" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
         <v>782</v>
       </c>
@@ -5490,7 +5499,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>783</v>
       </c>
@@ -5513,7 +5522,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="27" spans="1:7" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" s="12" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
         <v>791</v>
       </c>
@@ -5521,7 +5530,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>792</v>
       </c>
@@ -5529,7 +5538,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="29" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
         <v>793</v>
       </c>
@@ -5543,7 +5552,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>794</v>
       </c>
@@ -5570,15 +5579,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16196D24-437F-4113-984C-E1E07E6FEFBB}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -5595,7 +5604,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -5623,18 +5632,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A4B5976-09F6-46A1-AF3B-E9A8DFB4EAF3}">
   <dimension ref="A1:G68"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.109375" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.140625" customWidth="1"/>
     <col min="7" max="7" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -5651,7 +5660,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -5668,7 +5677,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -5685,7 +5694,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -5702,7 +5711,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -5719,7 +5728,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -5736,7 +5745,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>41</v>
       </c>
@@ -5753,7 +5762,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>46</v>
       </c>
@@ -5770,7 +5779,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -5793,7 +5802,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -5816,7 +5825,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -5824,7 +5833,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>64</v>
       </c>
@@ -5832,7 +5841,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -5852,7 +5861,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>70</v>
       </c>
@@ -5872,7 +5881,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>15</v>
       </c>
@@ -5880,7 +5889,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>85</v>
       </c>
@@ -5888,7 +5897,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>15</v>
       </c>
@@ -5905,7 +5914,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>89</v>
       </c>
@@ -5922,7 +5931,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="28" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>15</v>
       </c>
@@ -5936,7 +5945,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>96</v>
       </c>
@@ -5950,7 +5959,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>15</v>
       </c>
@@ -5967,7 +5976,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>102</v>
       </c>
@@ -5984,7 +5993,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="34" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>15</v>
       </c>
@@ -6001,7 +6010,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>110</v>
       </c>
@@ -6018,7 +6027,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="37" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>15</v>
       </c>
@@ -6035,7 +6044,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>118</v>
       </c>
@@ -6052,7 +6061,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="40" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>15</v>
       </c>
@@ -6069,7 +6078,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>126</v>
       </c>
@@ -6086,7 +6095,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="43" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>15</v>
       </c>
@@ -6106,7 +6115,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>134</v>
       </c>
@@ -6126,7 +6135,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
@@ -6149,7 +6158,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>144</v>
       </c>
@@ -6172,7 +6181,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>15</v>
       </c>
@@ -6189,7 +6198,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>155</v>
       </c>
@@ -6206,7 +6215,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="52" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>15</v>
       </c>
@@ -6220,7 +6229,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>163</v>
       </c>
@@ -6234,7 +6243,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="55" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>15</v>
       </c>
@@ -6251,7 +6260,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>169</v>
       </c>
@@ -6268,7 +6277,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="58" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>15</v>
       </c>
@@ -6285,7 +6294,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>177</v>
       </c>
@@ -6302,7 +6311,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="61" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>15</v>
       </c>
@@ -6316,7 +6325,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>184</v>
       </c>
@@ -6330,7 +6339,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="64" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>15</v>
       </c>
@@ -6347,7 +6356,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>187</v>
       </c>
@@ -6364,7 +6373,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="67" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>15</v>
       </c>
@@ -6381,7 +6390,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>195</v>
       </c>
@@ -6415,15 +6424,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B476B142-4B93-4B5F-AFDD-C5C6F475C99C}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.5546875" customWidth="1"/>
-    <col min="3" max="3" width="26.21875" customWidth="1"/>
-    <col min="4" max="4" width="28.77734375" customWidth="1"/>
-    <col min="5" max="5" width="31.44140625" customWidth="1"/>
+    <col min="2" max="2" width="23.5703125" customWidth="1"/>
+    <col min="3" max="3" width="26.28515625" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
+    <col min="5" max="5" width="31.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -6440,7 +6449,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>204</v>
       </c>
@@ -6457,7 +6466,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -6474,7 +6483,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>212</v>
       </c>
@@ -6491,7 +6500,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -6508,7 +6517,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>220</v>
       </c>
@@ -6525,7 +6534,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
@@ -6542,7 +6551,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>227</v>
       </c>
@@ -6567,17 +6576,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58630B64-2EDF-4356-94B8-66DDB845E6F8}">
   <dimension ref="A1:G38"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="36.88671875" customWidth="1"/>
-    <col min="4" max="4" width="37.5546875" customWidth="1"/>
-    <col min="5" max="5" width="39.21875" customWidth="1"/>
-    <col min="6" max="6" width="39.77734375" customWidth="1"/>
+    <col min="3" max="3" width="36.85546875" customWidth="1"/>
+    <col min="4" max="4" width="37.5703125" customWidth="1"/>
+    <col min="5" max="5" width="39.28515625" customWidth="1"/>
+    <col min="6" max="6" width="39.7109375" customWidth="1"/>
     <col min="7" max="7" width="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -6591,7 +6600,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>245</v>
       </c>
@@ -6605,7 +6614,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -6619,7 +6628,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>246</v>
       </c>
@@ -6633,7 +6642,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -6647,7 +6656,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>244</v>
       </c>
@@ -6661,7 +6670,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
@@ -6678,7 +6687,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>249</v>
       </c>
@@ -6695,7 +6704,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>251</v>
       </c>
@@ -6718,7 +6727,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>255</v>
       </c>
@@ -6741,7 +6750,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>251</v>
       </c>
@@ -6764,7 +6773,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>259</v>
       </c>
@@ -6787,7 +6796,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -6810,7 +6819,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>265</v>
       </c>
@@ -6833,7 +6842,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="22" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>15</v>
       </c>
@@ -6850,7 +6859,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>273</v>
       </c>
@@ -6867,7 +6876,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="25" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>15</v>
       </c>
@@ -6884,7 +6893,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>280</v>
       </c>
@@ -6901,7 +6910,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="28" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>15</v>
       </c>
@@ -6918,7 +6927,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>286</v>
       </c>
@@ -6935,7 +6944,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="31" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>251</v>
       </c>
@@ -6958,7 +6967,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>291</v>
       </c>
@@ -6981,7 +6990,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="34" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>15</v>
       </c>
@@ -6998,7 +7007,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>297</v>
       </c>
@@ -7015,7 +7024,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="37" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>15</v>
       </c>
@@ -7038,7 +7047,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>305</v>
       </c>
@@ -7075,15 +7084,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77AFD7FA-CE31-4CAB-9D77-EB9A0F5923D7}">
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="65.6640625" customWidth="1"/>
-    <col min="3" max="3" width="30.21875" customWidth="1"/>
-    <col min="4" max="4" width="33.88671875" customWidth="1"/>
-    <col min="5" max="6" width="40.21875" customWidth="1"/>
+    <col min="2" max="2" width="65.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" customWidth="1"/>
+    <col min="5" max="6" width="40.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -7100,7 +7109,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>245</v>
       </c>
@@ -7117,7 +7126,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -7134,7 +7143,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>322</v>
       </c>
@@ -7151,7 +7160,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -7168,7 +7177,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>328</v>
       </c>
@@ -7185,7 +7194,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
@@ -7202,7 +7211,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>255</v>
       </c>
@@ -7219,7 +7228,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -7236,7 +7245,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>339</v>
       </c>
@@ -7253,7 +7262,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>251</v>
       </c>
@@ -7270,7 +7279,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>349</v>
       </c>
@@ -7287,7 +7296,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="19" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -7307,7 +7316,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>353</v>
       </c>
@@ -7327,7 +7336,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="22" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>15</v>
       </c>
@@ -7344,7 +7353,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>360</v>
       </c>
@@ -7361,7 +7370,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="25" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>15</v>
       </c>
@@ -7378,7 +7387,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>366</v>
       </c>
@@ -7395,7 +7404,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="28" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>15</v>
       </c>
@@ -7412,7 +7421,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>376</v>
       </c>
@@ -7429,7 +7438,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="31" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>15</v>
       </c>
@@ -7446,7 +7455,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>380</v>
       </c>

</xml_diff>